<commit_message>
chore: add UTF-8 BOM to 13 SCL files
</commit_message>
<xml_diff>
--- a/Constant.xlsx
+++ b/Constant.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="263">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -133,67 +133,91 @@
     <t xml:space="preserve">Зупинити механізм</t>
   </si>
   <si>
+    <t xml:space="preserve">FLT_NONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Немає аварії</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_BREAKER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Аварія автомата захисту (BIT0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_OVERFLOW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Аварія переповнення (BIT1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_NO_RUNFB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Немає зворотного зв'язку роботи тахо (BIT2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">FLT_ALINGMENT</t>
   </si>
   <si>
-    <t xml:space="preserve">Word</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аварія вирівнювання (норія)</t>
+    <t xml:space="preserve">Аварія вирівнювання норія (BIT3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_NO_FEEDBACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Немає зворотного зв'язку контактора (BIT4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_GATE_MOVE_TIMEOUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Таймаут переміщення засувки (BIT5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_GATE_POS_UNKNOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Невідома позиція засувки після переміщення (BIT6)</t>
   </si>
   <si>
     <t xml:space="preserve">FLT_BOTH_SENSORS</t>
   </si>
   <si>
-    <t xml:space="preserve">Обидва кінцеві датчики активні одночасно (засувка)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_BREAKER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аварія автомата захисту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_GATE_MOVE_TIMEOUT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Таймаут переміщення засувки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_GATE_POS_UNKNOWN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Невідома позиція засувки після переміщення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_NO_FEEDBACK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Немає зворотного зв'язку контактора (редлер/норія/вентилятор/сепаратор)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_NO_RUNFB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Немає зворотного зв'язку роботи (норія/редлер/вентилятор)</t>
+    <t xml:space="preserve">Обидва кінцеві датчики активні одночасно засувка (BIT7)</t>
   </si>
   <si>
     <t xml:space="preserve">FLT_STOP_TIMEOUT</t>
   </si>
   <si>
-    <t xml:space="preserve">Таймаут вибігу при зупинці (редлер/норія/вентилятор/сепаратор/фідер)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_NONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Немає аварії</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_OVERFLOW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аварія переповнення</t>
+    <t xml:space="preserve">Таймаут вибігу при зупинці (BIT8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_VALVE_MOVE_TIMEOUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Таймаут переміщення клапана (BIT9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_VALVE_POS_UNKNOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Невідома позиція клапана після переміщення (BIT10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_VALVE_MULTIPLE_POS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кілька датчиків позиції клапана активні (BIT11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLT_INTERLOCK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Блокування (BIT12)</t>
   </si>
   <si>
     <t xml:space="preserve">GATE_AT_POS0</t>
@@ -739,9 +763,6 @@
     <t xml:space="preserve">ROUTE_MAX_STEPS</t>
   </si>
   <si>
-    <t xml:space="preserve">FLT_INTERLOCK</t>
-  </si>
-  <si>
     <t xml:space="preserve">ROUTE_STS_LOCKING</t>
   </si>
   <si>
@@ -769,18 +790,6 @@
     <t xml:space="preserve">Таймаут невизначеної позиції клапана (мс)</t>
   </si>
   <si>
-    <t xml:space="preserve">FLT_VALVE_MOVE_TIMEOUT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Таймаут переміщення клапана</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_VALVE_POS_UNKNOWN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Невідома позиція клапана після переміщення</t>
-  </si>
-  <si>
     <t xml:space="preserve">TYPE_Receiving_PIT</t>
   </si>
   <si>
@@ -800,9 +809,6 @@
   </si>
   <si>
     <t xml:space="preserve">центр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLT_VALVE_MULTIPLE_POS</t>
   </si>
 </sst>
 </file>
@@ -1012,14 +1018,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="64.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="56.21"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1305,7 +1311,7 @@
         <v>38</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>39</v>
@@ -1322,7 +1328,7 @@
         <v>38</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>41</v>
@@ -1339,7 +1345,7 @@
         <v>38</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>43</v>
@@ -1356,7 +1362,7 @@
         <v>38</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>45</v>
@@ -1373,7 +1379,7 @@
         <v>38</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>47</v>
@@ -1390,7 +1396,7 @@
         <v>38</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>49</v>
@@ -1407,7 +1413,7 @@
         <v>38</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>51</v>
@@ -1424,7 +1430,7 @@
         <v>38</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>53</v>
@@ -1441,7 +1447,7 @@
         <v>38</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>55</v>
@@ -1458,7 +1464,7 @@
         <v>38</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>10</v>
+        <v>256</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>57</v>
@@ -1472,78 +1478,78 @@
         <v>6</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>512</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>4096</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="D31" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>68</v>
@@ -1557,10 +1563,10 @@
         <v>6</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>70</v>
@@ -1574,10 +1580,10 @@
         <v>6</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>72</v>
@@ -1591,10 +1597,10 @@
         <v>6</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>74</v>
@@ -1608,10 +1614,10 @@
         <v>6</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>76</v>
@@ -1625,10 +1631,10 @@
         <v>6</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>78</v>
@@ -1645,7 +1651,7 @@
         <v>7</v>
       </c>
       <c r="D37" s="1" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>80</v>
@@ -1659,78 +1665,78 @@
         <v>6</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="D38" s="1" t="n">
-        <v>304</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D39" s="1" t="n">
-        <v>303</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D40" s="1" t="n">
-        <v>301</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D41" s="1" t="n">
-        <v>305</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="D42" s="1" t="n">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>91</v>
@@ -1744,10 +1750,10 @@
         <v>6</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D43" s="1" t="n">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>93</v>
@@ -1761,10 +1767,10 @@
         <v>6</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D44" s="1" t="n">
-        <v>200</v>
+        <v>301</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>95</v>
@@ -1778,10 +1784,10 @@
         <v>6</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D45" s="1" t="n">
-        <v>203</v>
+        <v>305</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>97</v>
@@ -1795,10 +1801,10 @@
         <v>6</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D46" s="1" t="n">
-        <v>202</v>
+        <v>302</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>99</v>
@@ -1812,10 +1818,10 @@
         <v>6</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D47" s="1" t="n">
-        <v>201</v>
+        <v>306</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>101</v>
@@ -1829,10 +1835,10 @@
         <v>6</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D48" s="1" t="n">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>103</v>
@@ -1846,10 +1852,10 @@
         <v>6</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D49" s="1" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>105</v>
@@ -1863,10 +1869,10 @@
         <v>6</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D50" s="1" t="n">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>107</v>
@@ -1880,10 +1886,10 @@
         <v>6</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D51" s="1" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>109</v>
@@ -1897,10 +1903,10 @@
         <v>6</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D52" s="1" t="n">
-        <v>8</v>
+        <v>205</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>111</v>
@@ -1914,10 +1920,10 @@
         <v>6</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D53" s="1" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>113</v>
@@ -1931,10 +1937,10 @@
         <v>6</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D54" s="1" t="n">
-        <v>7</v>
+        <v>206</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>115</v>
@@ -1948,10 +1954,10 @@
         <v>6</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D55" s="1" t="n">
-        <v>4</v>
+        <v>207</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>117</v>
@@ -1965,10 +1971,10 @@
         <v>6</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D56" s="1" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>119</v>
@@ -1982,10 +1988,10 @@
         <v>6</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D57" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>121</v>
@@ -1999,10 +2005,10 @@
         <v>6</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>123</v>
@@ -2016,10 +2022,10 @@
         <v>6</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="D59" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>125</v>
@@ -2033,7 +2039,7 @@
         <v>6</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="D60" s="1" t="n">
         <v>2</v>
@@ -2050,10 +2056,10 @@
         <v>6</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>129</v>
@@ -2067,10 +2073,10 @@
         <v>6</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="D62" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>131</v>
@@ -2104,7 +2110,7 @@
         <v>7</v>
       </c>
       <c r="D64" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>135</v>
@@ -2121,7 +2127,7 @@
         <v>7</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>137</v>
@@ -2138,7 +2144,7 @@
         <v>7</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>139</v>
@@ -2155,7 +2161,7 @@
         <v>7</v>
       </c>
       <c r="D67" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>141</v>
@@ -2172,7 +2178,7 @@
         <v>7</v>
       </c>
       <c r="D68" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>143</v>
@@ -2189,7 +2195,7 @@
         <v>7</v>
       </c>
       <c r="D69" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>145</v>
@@ -2206,7 +2212,7 @@
         <v>7</v>
       </c>
       <c r="D70" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>147</v>
@@ -2223,7 +2229,7 @@
         <v>7</v>
       </c>
       <c r="D71" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>149</v>
@@ -2240,7 +2246,7 @@
         <v>7</v>
       </c>
       <c r="D72" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>151</v>
@@ -2254,10 +2260,10 @@
         <v>6</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="D73" s="1" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>153</v>
@@ -2271,10 +2277,10 @@
         <v>6</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="D74" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>155</v>
@@ -2288,10 +2294,10 @@
         <v>6</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="D75" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>157</v>
@@ -2305,146 +2311,146 @@
         <v>6</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="D76" s="1" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D77" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D78" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D79" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="D80" s="1" t="n">
-        <v>5000</v>
+        <v>11</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>167</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D81" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D81" s="1" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D82" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D82" s="1" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D83" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D83" s="1" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B84" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="D84" s="1" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>175</v>
@@ -2458,7 +2464,7 @@
         <v>6</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D85" s="1" t="n">
         <v>2000</v>
@@ -2475,7 +2481,7 @@
         <v>6</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D86" s="1" t="n">
         <v>10000</v>
@@ -2492,10 +2498,10 @@
         <v>6</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D87" s="1" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>181</v>
@@ -2509,10 +2515,10 @@
         <v>6</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D88" s="1" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>183</v>
@@ -2526,7 +2532,7 @@
         <v>6</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D89" s="1" t="n">
         <v>2000</v>
@@ -2543,7 +2549,7 @@
         <v>6</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D90" s="1" t="n">
         <v>10000</v>
@@ -2560,7 +2566,7 @@
         <v>6</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D91" s="1" t="n">
         <v>2000</v>
@@ -2577,7 +2583,7 @@
         <v>6</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D92" s="1" t="n">
         <v>5000</v>
@@ -2594,10 +2600,10 @@
         <v>6</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D93" s="1" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>193</v>
@@ -2611,10 +2617,10 @@
         <v>6</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D94" s="1" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="E94" s="1" t="s">
         <v>195</v>
@@ -2628,10 +2634,10 @@
         <v>6</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D95" s="1" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>197</v>
@@ -2645,7 +2651,7 @@
         <v>6</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D96" s="1" t="n">
         <v>5000</v>
@@ -2662,10 +2668,10 @@
         <v>6</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D97" s="1" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>201</v>
@@ -2679,10 +2685,10 @@
         <v>6</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D98" s="1" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>203</v>
@@ -2696,10 +2702,10 @@
         <v>6</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D99" s="1" t="n">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>205</v>
@@ -2713,10 +2719,10 @@
         <v>6</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D100" s="1" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E100" s="1" t="s">
         <v>207</v>
@@ -2730,10 +2736,10 @@
         <v>6</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D101" s="1" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>209</v>
@@ -2747,10 +2753,10 @@
         <v>6</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D102" s="1" t="n">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="E102" s="1" t="s">
         <v>211</v>
@@ -2764,7 +2770,7 @@
         <v>6</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D103" s="1" t="n">
         <v>3000</v>
@@ -2781,10 +2787,10 @@
         <v>6</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D104" s="1" t="n">
-        <v>4</v>
+        <v>3000</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>215</v>
@@ -2798,10 +2804,10 @@
         <v>6</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D105" s="1" t="n">
-        <v>3</v>
+        <v>5000</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>217</v>
@@ -2815,10 +2821,10 @@
         <v>6</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D106" s="1" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>219</v>
@@ -2832,10 +2838,10 @@
         <v>6</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D107" s="1" t="n">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>221</v>
@@ -2852,7 +2858,7 @@
         <v>7</v>
       </c>
       <c r="D108" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>223</v>
@@ -2869,7 +2875,7 @@
         <v>7</v>
       </c>
       <c r="D109" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E109" s="1" t="s">
         <v>225</v>
@@ -2886,7 +2892,7 @@
         <v>7</v>
       </c>
       <c r="D110" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E110" s="1" t="s">
         <v>227</v>
@@ -2903,7 +2909,7 @@
         <v>7</v>
       </c>
       <c r="D111" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E111" s="1" t="s">
         <v>229</v>
@@ -2920,7 +2926,7 @@
         <v>7</v>
       </c>
       <c r="D112" s="1" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E112" s="1" t="s">
         <v>231</v>
@@ -2937,7 +2943,7 @@
         <v>7</v>
       </c>
       <c r="D113" s="1" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E113" s="1" t="s">
         <v>233</v>
@@ -2954,7 +2960,7 @@
         <v>7</v>
       </c>
       <c r="D114" s="1" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E114" s="1" t="s">
         <v>235</v>
@@ -2971,7 +2977,7 @@
         <v>7</v>
       </c>
       <c r="D115" s="1" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>237</v>
@@ -2988,43 +2994,49 @@
         <v>7</v>
       </c>
       <c r="D116" s="1" t="n">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>74</v>
+        <v>239</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="D117" s="1" t="n">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="D118" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>6</v>
@@ -3033,15 +3045,15 @@
         <v>7</v>
       </c>
       <c r="D119" s="1" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>6</v>
@@ -3050,27 +3062,27 @@
         <v>7</v>
       </c>
       <c r="D120" s="1" t="n">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>244</v>
+        <v>82</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
-        <v>245</v>
+        <v>64</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>166</v>
+        <v>38</v>
       </c>
       <c r="D121" s="1" t="n">
-        <v>15000</v>
+        <v>4096</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>246</v>
+        <v>65</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3081,61 +3093,61 @@
         <v>6</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="D122" s="1" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E122" s="1" t="s">
-        <v>248</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D123" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E123" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="B123" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D123" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="E123" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E124" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C124" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D124" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D125" s="1" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E125" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D125" s="1" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3146,10 +3158,10 @@
         <v>6</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D126" s="1" t="n">
-        <v>3</v>
+        <v>15000</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>255</v>
@@ -3157,79 +3169,119 @@
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
-        <v>256</v>
+        <v>58</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="D127" s="1" t="n">
-        <v>4</v>
+        <v>512</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>257</v>
+        <v>59</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
-        <v>258</v>
+        <v>60</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="D128" s="1" t="n">
-        <v>5</v>
+        <v>1024</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>259</v>
+        <v>61</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D129" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D130" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D131" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E131" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B129" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C129" s="1" t="s">
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D132" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D129" s="1" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="0"/>
-      <c r="B130" s="0"/>
-      <c r="C130" s="0"/>
-      <c r="D130" s="0"/>
-      <c r="E130" s="0"/>
-    </row>
-    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="0"/>
-      <c r="B131" s="0"/>
-      <c r="C131" s="0"/>
-      <c r="D131" s="0"/>
-      <c r="E131" s="0"/>
-    </row>
-    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="0"/>
-      <c r="B132" s="0"/>
-      <c r="C132" s="0"/>
-      <c r="D132" s="0"/>
-      <c r="E132" s="0"/>
-    </row>
-    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="0"/>
-      <c r="B133" s="0"/>
-      <c r="C133" s="0"/>
-      <c r="D133" s="0"/>
-      <c r="E133" s="0"/>
+      <c r="D133" s="1" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="0"/>
@@ -3244,6 +3296,34 @@
       <c r="C135" s="0"/>
       <c r="D135" s="0"/>
       <c r="E135" s="0"/>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="0"/>
+      <c r="B136" s="0"/>
+      <c r="C136" s="0"/>
+      <c r="D136" s="0"/>
+      <c r="E136" s="0"/>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="0"/>
+      <c r="B137" s="0"/>
+      <c r="C137" s="0"/>
+      <c r="D137" s="0"/>
+      <c r="E137" s="0"/>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="0"/>
+      <c r="B138" s="0"/>
+      <c r="C138" s="0"/>
+      <c r="D138" s="0"/>
+      <c r="E138" s="0"/>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="0"/>
+      <c r="B139" s="0"/>
+      <c r="C139" s="0"/>
+      <c r="D139" s="0"/>
+      <c r="E139" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>